<commit_message>
Add Strategy review doc, update cost model with Product Summary sheet
Strategy: kept pwin-win-strategy-review.docx as design input (four-phase
model, five elicitation dimensions, reference library architecture).
Removed SKILL.md and win-strategy.md — subsets of the docx, written
before MCP architecture superseded the /pwin: command pattern.

Cost model: added Sheet 6 (Product Cost Summary) breaking out Qualify,
Execution, and Verdict API costs side by side with combined portfolio
scaling scenarios.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/pwin-platform/docs/BidEquity_API_Cost_Model.xlsx
+++ b/pwin-platform/docs/BidEquity_API_Cost_Model.xlsx
@@ -12,7 +12,8 @@
     <sheet name="Client Portfolio" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Cost Reduction Levers" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Verdict Product" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Assumptions" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Product Cost Summary" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Assumptions" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -138,7 +139,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -205,6 +206,7 @@
     <xf numFmtId="166" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
@@ -5134,6 +5136,827 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:F55"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="20" t="inlineStr">
+        <is>
+          <t>BidEquity Platform — API Cost by Product</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="2" t="n"/>
+      <c r="D1" s="2" t="n"/>
+      <c r="E1" s="2" t="n"/>
+      <c r="F1" s="2" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="30" t="inlineStr">
+        <is>
+          <t>All costs are Claude API token costs only. Consultant time, infrastructure, and overheads are excluded.</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="n"/>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="2" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="17" t="inlineStr">
+        <is>
+          <t>PWIN QUALIFY</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Step</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Invocations</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Input Tokens</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Output Tokens</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>Cost (USD)</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="22" t="inlineStr">
+        <is>
+          <t>AI Assurance Review (per question)</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="C6" s="6" t="n">
+        <v>60000</v>
+      </c>
+      <c r="D6" s="6" t="n">
+        <v>19200</v>
+      </c>
+      <c r="E6" s="7" t="n">
+        <v>0.468</v>
+      </c>
+      <c r="F6" s="9" t="inlineStr">
+        <is>
+          <t>System prompt + question + evidence + rubric + sector context. Currently calls Claude API directly from browser.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="22" t="inlineStr">
+        <is>
+          <t>Full Qualification Report</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C7" s="6" t="n">
+        <v>5000</v>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>2000</v>
+      </c>
+      <c r="E7" s="7" t="n">
+        <v>0.045</v>
+      </c>
+      <c r="F7" s="9" t="inlineStr">
+        <is>
+          <t>Synthesises all 24 reviews into overall assessment with PWIN score.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="22" t="inlineStr">
+        <is>
+          <t>PWIN Score Calculation</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="C8" s="6" t="n">
+        <v>9000</v>
+      </c>
+      <c r="D8" s="6" t="n">
+        <v>1500</v>
+      </c>
+      <c r="E8" s="7" t="n">
+        <v>0.0495</v>
+      </c>
+      <c r="F8" s="9" t="inlineStr">
+        <is>
+          <t>At initial assessment, post-review, and final. Lightweight calculation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="15" t="inlineStr">
+        <is>
+          <t>Qualify Total per Pursuit</t>
+        </is>
+      </c>
+      <c r="E10" s="16" t="n">
+        <v>0.5625</v>
+      </c>
+      <c r="F10" s="15" t="inlineStr">
+        <is>
+          <t>GBP: £0.44</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="17" t="inlineStr">
+        <is>
+          <t>PWIN EXECUTION (Bid Lifecycle)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Phase</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Skills</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>Invocations</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>Cost (USD)</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="22" t="inlineStr">
+        <is>
+          <t>Pre-Bid</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="C14" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="D14" s="8" t="n">
+        <v>0.4485</v>
+      </c>
+      <c r="E14" s="9" t="inlineStr">
+        <is>
+          <t>Client profiling, sector scanning, incumbent, competitors, stakeholders — REUSABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="22" t="inlineStr">
+        <is>
+          <t>ITT Receipt</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="C15" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="D15" s="8" t="n">
+        <v>0.5475</v>
+      </c>
+      <c r="E15" s="9" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="22" t="inlineStr">
+        <is>
+          <t>Strategy</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="C16" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="D16" s="8" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="E16" s="9" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="22" t="inlineStr">
+        <is>
+          <t>Solution</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="C17" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="D17" s="8" t="n">
+        <v>1.71</v>
+      </c>
+      <c r="E17" s="9" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="22" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="C18" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="D18" s="8" t="n">
+        <v>1.0725</v>
+      </c>
+      <c r="E18" s="9" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="22" t="inlineStr">
+        <is>
+          <t>Production</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="C19" s="6" t="n">
+        <v>36</v>
+      </c>
+      <c r="D19" s="8" t="n">
+        <v>3.78</v>
+      </c>
+      <c r="E19" s="9" t="inlineStr">
+        <is>
+          <t>Drafting (10×), Formatting (10×), Win theme audit (3×), Review trajectory (3×)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="22" t="inlineStr">
+        <is>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="C20" s="6" t="n">
+        <v>50</v>
+      </c>
+      <c r="D20" s="8" t="n">
+        <v>5.325</v>
+      </c>
+      <c r="E20" s="9" t="inlineStr">
+        <is>
+          <t>Standup (30×), Timeline (8×), Compliance (4×), Effort reforecast (4×), Bid cost (4×)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="22" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="C21" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="D21" s="8" t="n">
+        <v>1.5825</v>
+      </c>
+      <c r="E21" s="9" t="inlineStr">
+        <is>
+          <t>Gate readiness (5×), Governance packs (5×), Stakeholder risk (2×), Risk/pricing (1×)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="22" t="inlineStr">
+        <is>
+          <t>Mid-Bid</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="C22" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="D22" s="8" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="E22" s="9" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="22" t="inlineStr">
+        <is>
+          <t>Pre-Submit</t>
+        </is>
+      </c>
+      <c r="B23" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C23" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D23" s="8" t="n">
+        <v>0.1275</v>
+      </c>
+      <c r="E23" s="9" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="22" t="inlineStr">
+        <is>
+          <t>Post-Submit</t>
+        </is>
+      </c>
+      <c r="B24" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C24" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D24" s="8" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="E24" s="9" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="15" t="inlineStr">
+        <is>
+          <t>Execution Total per Opportunity</t>
+        </is>
+      </c>
+      <c r="D26" s="16" t="n">
+        <v>15.92849999999999</v>
+      </c>
+      <c r="E26" s="15" t="inlineStr">
+        <is>
+          <t>GBP: £12.58</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="17" t="inlineStr">
+        <is>
+          <t>BIDEQUITY VERDICT (Post-Loss Review)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Step</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>Cost (USD)</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="22" t="inlineStr">
+        <is>
+          <t>Document ingestion (ITT + proposal)</t>
+        </is>
+      </c>
+      <c r="B30" s="8" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="C30" s="9" t="inlineStr">
+        <is>
+          <t>2 skills: ITT extraction + proposal parsing</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="22" t="inlineStr">
+        <is>
+          <t>8 domain assessments (Pass 1)</t>
+        </is>
+      </c>
+      <c r="B31" s="8" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="C31" s="9" t="inlineStr">
+        <is>
+          <t>8 forensic domain skills</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="22" t="inlineStr">
+        <is>
+          <t>Independent scoring (8 sections)</t>
+        </is>
+      </c>
+      <c r="B32" s="8" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="C32" s="9" t="inlineStr">
+        <is>
+          <t>Per-section scoring against evaluation criteria</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="22" t="inlineStr">
+        <is>
+          <t>Traceability analysis</t>
+        </is>
+      </c>
+      <c r="B33" s="8" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="C33" s="9" t="inlineStr">
+        <is>
+          <t>Cross-artefact chain mapping</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="22" t="inlineStr">
+        <is>
+          <t>Pass 2 re-assessment (post-interview)</t>
+        </is>
+      </c>
+      <c r="B34" s="8" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="C34" s="9" t="inlineStr">
+        <is>
+          <t>8 domains re-run with enriched data</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="22" t="inlineStr">
+        <is>
+          <t>Report assembly</t>
+        </is>
+      </c>
+      <c r="B35" s="8" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="C35" s="9" t="inlineStr">
+        <is>
+          <t>Consolidates all findings into Verdict Report</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="15" t="inlineStr">
+        <is>
+          <t>Verdict Total per Engagement</t>
+        </is>
+      </c>
+      <c r="B37" s="16" t="n">
+        <v>2.53</v>
+      </c>
+      <c r="C37" s="15" t="inlineStr">
+        <is>
+          <t>GBP: £2.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="17" t="inlineStr">
+        <is>
+          <t>COMBINED COST SUMMARY</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>Cost per Use (USD)</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="inlineStr">
+        <is>
+          <t>Cost per Use (GBP)</t>
+        </is>
+      </c>
+      <c r="D41" s="4" t="inlineStr">
+        <is>
+          <t>Price to Client</t>
+        </is>
+      </c>
+      <c r="E41" s="4" t="inlineStr">
+        <is>
+          <t>API as % Price</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="22" t="inlineStr">
+        <is>
+          <t>Qualify (per pursuit)</t>
+        </is>
+      </c>
+      <c r="B42" s="8" t="n">
+        <v>0.5625</v>
+      </c>
+      <c r="C42" s="8" t="n">
+        <v>0.444375</v>
+      </c>
+      <c r="D42" s="22" t="inlineStr">
+        <is>
+          <t>Included in Core/Command</t>
+        </is>
+      </c>
+      <c r="E42" s="5" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="22" t="inlineStr">
+        <is>
+          <t>Execution (per opportunity)</t>
+        </is>
+      </c>
+      <c r="B43" s="8" t="n">
+        <v>15.92849999999999</v>
+      </c>
+      <c r="C43" s="8" t="n">
+        <v>12.583515</v>
+      </c>
+      <c r="D43" s="22" t="inlineStr">
+        <is>
+          <t>Included in Core/Command</t>
+        </is>
+      </c>
+      <c r="E43" s="5" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="22" t="inlineStr">
+        <is>
+          <t>Qualify + Execution combined</t>
+        </is>
+      </c>
+      <c r="B44" s="8" t="n">
+        <v>16.49099999999999</v>
+      </c>
+      <c r="C44" s="8" t="n">
+        <v>13.02788999999999</v>
+      </c>
+      <c r="D44" s="22" t="inlineStr">
+        <is>
+          <t>£80-500k/yr (Core/Command)</t>
+        </is>
+      </c>
+      <c r="E44" s="23" t="n">
+        <v>0.0001628486249999999</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="22" t="inlineStr">
+        <is>
+          <t>Verdict Single</t>
+        </is>
+      </c>
+      <c r="B45" s="8" t="n">
+        <v>2.53</v>
+      </c>
+      <c r="C45" s="8" t="n">
+        <v>1.9987</v>
+      </c>
+      <c r="D45" s="22" t="inlineStr">
+        <is>
+          <t>£2,000</t>
+        </is>
+      </c>
+      <c r="E45" s="23" t="n">
+        <v>0.00099935</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="22" t="inlineStr">
+        <is>
+          <t>Verdict Portfolio (×3)</t>
+        </is>
+      </c>
+      <c r="B46" s="8" t="n">
+        <v>7.59</v>
+      </c>
+      <c r="C46" s="8" t="n">
+        <v>5.9961</v>
+      </c>
+      <c r="D46" s="22" t="inlineStr">
+        <is>
+          <t>£5,000</t>
+        </is>
+      </c>
+      <c r="E46" s="23" t="n">
+        <v>0.00119922</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="17" t="inlineStr">
+        <is>
+          <t>ANNUAL SCALING SCENARIO</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>Client Scenario</t>
+        </is>
+      </c>
+      <c r="B50" s="4" t="inlineStr">
+        <is>
+          <t>Opps/Year</t>
+        </is>
+      </c>
+      <c r="C50" s="4" t="inlineStr">
+        <is>
+          <t>API/Year (GBP)</t>
+        </is>
+      </c>
+      <c r="D50" s="4" t="inlineStr">
+        <is>
+          <t>Revenue/Year</t>
+        </is>
+      </c>
+      <c r="E50" s="4" t="inlineStr">
+        <is>
+          <t>API as % Revenue</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="22" t="inlineStr">
+        <is>
+          <t>1 Core client, 5 opps</t>
+        </is>
+      </c>
+      <c r="B51" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="C51" s="8" t="n">
+        <v>65.13944999999997</v>
+      </c>
+      <c r="D51" s="8" t="n">
+        <v>80000</v>
+      </c>
+      <c r="E51" s="23" t="n">
+        <v>0.0008142431249999996</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="22" t="inlineStr">
+        <is>
+          <t>1 Command client, 15 opps</t>
+        </is>
+      </c>
+      <c r="B52" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="C52" s="8" t="n">
+        <v>195.4183499999999</v>
+      </c>
+      <c r="D52" s="8" t="n">
+        <v>250000</v>
+      </c>
+      <c r="E52" s="23" t="n">
+        <v>0.0007816733999999997</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="22" t="inlineStr">
+        <is>
+          <t>5 Core + 2 Command clients</t>
+        </is>
+      </c>
+      <c r="B53" s="6" t="n">
+        <v>55</v>
+      </c>
+      <c r="C53" s="8" t="n">
+        <v>716.5339499999997</v>
+      </c>
+      <c r="D53" s="8" t="n">
+        <v>900000</v>
+      </c>
+      <c r="E53" s="23" t="n">
+        <v>0.000796148833333333</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="22" t="inlineStr">
+        <is>
+          <t>10 Verdict Singles/year</t>
+        </is>
+      </c>
+      <c r="B54" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="C54" s="8" t="n">
+        <v>19.987</v>
+      </c>
+      <c r="D54" s="8" t="n">
+        <v>20000</v>
+      </c>
+      <c r="E54" s="23" t="n">
+        <v>0.00099935</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="22" t="inlineStr">
+        <is>
+          <t>Full portfolio: 5 Core + 2 Command + 10 Verdicts</t>
+        </is>
+      </c>
+      <c r="B55" s="6" t="n">
+        <v>65</v>
+      </c>
+      <c r="C55" s="8" t="n">
+        <v>736.5209499999996</v>
+      </c>
+      <c r="D55" s="8" t="n">
+        <v>920000</v>
+      </c>
+      <c r="E55" s="23" t="n">
+        <v>0.0008005662499999996</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:C19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -5168,7 +5991,7 @@
           <t>Pricing</t>
         </is>
       </c>
-      <c r="B4" s="30" t="inlineStr">
+      <c r="B4" s="31" t="inlineStr">
         <is>
           <t>Claude Sonnet 4: $3.00/M input tokens, $15.00/M output tokens</t>
         </is>
@@ -5180,7 +6003,7 @@
           <t>Pricing</t>
         </is>
       </c>
-      <c r="B5" s="30" t="inlineStr">
+      <c r="B5" s="31" t="inlineStr">
         <is>
           <t>Claude Haiku 4.5: $0.25/M input tokens, $1.25/M output tokens</t>
         </is>
@@ -5192,7 +6015,7 @@
           <t>Pricing</t>
         </is>
       </c>
-      <c r="B6" s="30" t="inlineStr">
+      <c r="B6" s="31" t="inlineStr">
         <is>
           <t>Claude Opus 4: $15.00/M input tokens, $75.00/M output tokens</t>
         </is>
@@ -5204,7 +6027,7 @@
           <t>Pricing</t>
         </is>
       </c>
-      <c r="B7" s="30" t="inlineStr">
+      <c r="B7" s="31" t="inlineStr">
         <is>
           <t>USD to GBP exchange rate: 0.79</t>
         </is>
@@ -5216,7 +6039,7 @@
           <t>Pricing</t>
         </is>
       </c>
-      <c r="B8" s="30" t="inlineStr">
+      <c r="B8" s="31" t="inlineStr">
         <is>
           <t>Prices are list rates — volume discounts may apply at scale</t>
         </is>
@@ -5228,7 +6051,7 @@
           <t>Token estimates</t>
         </is>
       </c>
-      <c r="B9" s="30" t="inlineStr">
+      <c r="B9" s="31" t="inlineStr">
         <is>
           <t>Based on live tests: Timeline Analysis (42,825 in / 2,097 out), Compliance Coverage (37,589 in / 1,856 out), ITT Extraction (21,260 in / 1,719 out)</t>
         </is>
@@ -5240,7 +6063,7 @@
           <t>Token estimates</t>
         </is>
       </c>
-      <c r="B10" s="30" t="inlineStr">
+      <c r="B10" s="31" t="inlineStr">
         <is>
           <t>Non-tested skills estimated by analogy to tested skills, adjusted for expected context size and output length</t>
         </is>
@@ -5252,7 +6075,7 @@
           <t>Token estimates</t>
         </is>
       </c>
-      <c r="B11" s="30" t="inlineStr">
+      <c r="B11" s="31" t="inlineStr">
         <is>
           <t>Multi-turn tool use adds ~20-30% overhead vs single-turn (tool call results returned to Claude)</t>
         </is>
@@ -5264,7 +6087,7 @@
           <t>Frequency</t>
         </is>
       </c>
-      <c r="B12" s="30" t="inlineStr">
+      <c r="B12" s="31" t="inlineStr">
         <is>
           <t>Medium bid (£25-100m) assumed as baseline: 10 response sections, 10-week duration, 5 governance gates</t>
         </is>
@@ -5276,7 +6099,7 @@
           <t>Frequency</t>
         </is>
       </c>
-      <c r="B13" s="30" t="inlineStr">
+      <c r="B13" s="31" t="inlineStr">
         <is>
           <t>Standup Priorities (Skill 3.7) at 30 calls/opp is the single highest-frequency skill — daily for 6 weeks</t>
         </is>
@@ -5288,7 +6111,7 @@
           <t>Frequency</t>
         </is>
       </c>
-      <c r="B14" s="30" t="inlineStr">
+      <c r="B14" s="31" t="inlineStr">
         <is>
           <t>Response Section Drafting (Skill 5.1) and Production Formatting (Skill 5.5) scale linearly with section count</t>
         </is>
@@ -5300,7 +6123,7 @@
           <t>Revenue</t>
         </is>
       </c>
-      <c r="B15" s="30" t="inlineStr">
+      <c r="B15" s="31" t="inlineStr">
         <is>
           <t>Core client revenue: £80-120k/year. Command client: £200-500k/year. Verdict Single: £2k, Portfolio: £5k</t>
         </is>
@@ -5312,7 +6135,7 @@
           <t>Consultant cost</t>
         </is>
       </c>
-      <c r="B16" s="30" t="inlineStr">
+      <c r="B16" s="31" t="inlineStr">
         <is>
           <t>Verdict consultant time: 1.5 days per Single (intake + interview + report review + debrief) at £800/day internal cost</t>
         </is>
@@ -5324,7 +6147,7 @@
           <t>Prompt caching</t>
         </is>
       </c>
-      <c r="B17" s="30" t="inlineStr">
+      <c r="B17" s="31" t="inlineStr">
         <is>
           <t>Anthropic prompt caching reduces cost of repeated system prompt by ~90%. Applicable when same system prompt is used across multiple calls in a session.</t>
         </is>
@@ -5336,7 +6159,7 @@
           <t>Pre-built intel</t>
         </is>
       </c>
-      <c r="B18" s="30" t="inlineStr">
+      <c r="B18" s="31" t="inlineStr">
         <is>
           <t>Client profiles and competitor dossiers, once built, eliminate the research cost for repeat clients. Build cost is a one-time investment via Claude Pro subscription or initial API call.</t>
         </is>
@@ -5348,7 +6171,7 @@
           <t>Scaling</t>
         </is>
       </c>
-      <c r="B19" s="30" t="inlineStr">
+      <c r="B19" s="31" t="inlineStr">
         <is>
           <t>Token usage scales with bid complexity (more sections = more drafting calls, more gates = more readiness calls) but NOT linearly — platform knowledge and pursuit context are fixed overhead.</t>
         </is>

</xml_diff>